<commit_message>
fixed ongoing session errors
</commit_message>
<xml_diff>
--- a/Data/CP_sessions_2023.xlsx
+++ b/Data/CP_sessions_2023.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/araavind/Desktop/Python Files/LEC-Opt/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52D8DFF6-E349-DF42-8981-0D8894E596B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD84DAF-913F-454C-9B4E-4A2A9028B54B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-1360" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-76800" yWindow="-1360" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CP1" sheetId="1" r:id="rId1"/>
@@ -118,16 +118,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -464,7 +461,7 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -508,7 +505,7 @@
         <v>44928.666666666657</v>
       </c>
       <c r="D3" s="2">
-        <v>44929.395833333343</v>
+        <v>44929.71875</v>
       </c>
       <c r="E3">
         <v>0.70981234760052381</v>
@@ -11092,7 +11089,7 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added function to create scenarios
</commit_message>
<xml_diff>
--- a/Data/CP_sessions_2023.xlsx
+++ b/Data/CP_sessions_2023.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/araavind/Desktop/Python Files/LEC-Opt/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD84DAF-913F-454C-9B4E-4A2A9028B54B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B19668-5852-5045-BC5B-DDE21C87ECF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-76800" yWindow="-1360" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -433,6 +433,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9" customWidth="1"/>
   </cols>
   <sheetData>
@@ -505,7 +506,7 @@
         <v>44928.666666666657</v>
       </c>
       <c r="D3" s="2">
-        <v>44929.71875</v>
+        <v>44929.46875</v>
       </c>
       <c r="E3">
         <v>0.70981234760052381</v>
@@ -531,7 +532,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="2">
-        <v>44929.864583333343</v>
+        <v>44929.864583333336</v>
       </c>
       <c r="D4" s="2">
         <v>44930.302083333343</v>

</xml_diff>